<commit_message>
actualizar error en muestra y ortografía
</commit_message>
<xml_diff>
--- a/fhir/ig/r2bo/0.3.0-draft/StructureDefinition-r2bo-muestra-biopsia.xlsx
+++ b/fhir/ig/r2bo/0.3.0-draft/StructureDefinition-r2bo-muestra-biopsia.xlsx
@@ -10,13 +10,13 @@
     <sheet name="Elements" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AM$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">Elements!$A$1:$AM$54</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2088" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1913" uniqueCount="377">
   <si>
     <t>Property</t>
   </si>
@@ -69,7 +69,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-20T12:25:24-04:00</t>
+    <t>2026-08-20T16:22:48-04:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -811,16 +811,31 @@
     <t>SPM-7</t>
   </si>
   <si>
-    <t>Specimen.collection.method.id</t>
-  </si>
-  <si>
-    <t>Specimen.collection.method.extension</t>
-  </si>
-  <si>
-    <t>Extension</t>
-  </si>
-  <si>
-    <t>An Extension</t>
+    <t>Specimen.collection.bodySite</t>
+  </si>
+  <si>
+    <t>Sitio anatómico de la colección</t>
+  </si>
+  <si>
+    <t>Anatomical location from which the specimen was collected (if subject is a patient). This is the target site.  This element is not used for environmental specimens.</t>
+  </si>
+  <si>
+    <t>If the use case requires  BodySite to be handled as a separate resource instead of an inline coded element (e.g. to identify and track separately)  then use the standard extension [bodySite](http://hl7.org/fhir/R4/extension-bodysite.html).</t>
+  </si>
+  <si>
+    <t>https://interoperabilidad.minsal.cl/fhir/ig/r2bo/ValueSet/r2bo-estructuras-anatomicas-VS</t>
+  </si>
+  <si>
+    <t>.targetSiteCode</t>
+  </si>
+  <si>
+    <t>SPM-8 and SPM-9</t>
+  </si>
+  <si>
+    <t>Specimen.collection.bodySite.id</t>
+  </si>
+  <si>
+    <t>Specimen.collection.bodySite.extension</t>
   </si>
   <si>
     <t xml:space="preserve">value:url}
@@ -833,23 +848,23 @@
     <t>open</t>
   </si>
   <si>
-    <t>Specimen.collection.method.extension:MetodoProcedimiento</t>
-  </si>
-  <si>
-    <t>MetodoProcedimiento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extension {https://interoperabilidad.minsal.cl/fhir/ig/r2bo/StructureDefinition/r2bo-extension-tipo-procedimientos-biopsias}
+    <t>Specimen.collection.bodySite.extension:CalificadorLateralidad</t>
+  </si>
+  <si>
+    <t>CalificadorLateralidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Extension {http://hl7.org/fhir/us/mcode/StructureDefinition/mcode-laterality-qualifier}
 </t>
   </si>
   <si>
-    <t>Método de procedimiento</t>
-  </si>
-  <si>
-    <t>Extensión que define los tipos de procedimientos al momento de extraer muestras de tejido</t>
-  </si>
-  <si>
-    <t>Specimen.collection.method.coding</t>
+    <t>Calificador para lateralidad para este sitio del cuerpo</t>
+  </si>
+  <si>
+    <t>Qualifier to specify laterality.</t>
+  </si>
+  <si>
+    <t>Specimen.collection.bodySite.coding</t>
   </si>
   <si>
     <t xml:space="preserve">Coding
@@ -877,7 +892,7 @@
     <t>C*E.1-8, C*E.10-22</t>
   </si>
   <si>
-    <t>Specimen.collection.method.text</t>
+    <t>Specimen.collection.bodySite.text</t>
   </si>
   <si>
     <t>Plain text representation of the concept</t>
@@ -899,55 +914,6 @@
   </si>
   <si>
     <t>C*E.9. But note many systems use C*E.2 for this</t>
-  </si>
-  <si>
-    <t>Specimen.collection.bodySite</t>
-  </si>
-  <si>
-    <t>Sitio anatómico de la colección</t>
-  </si>
-  <si>
-    <t>Anatomical location from which the specimen was collected (if subject is a patient). This is the target site.  This element is not used for environmental specimens.</t>
-  </si>
-  <si>
-    <t>If the use case requires  BodySite to be handled as a separate resource instead of an inline coded element (e.g. to identify and track separately)  then use the standard extension [bodySite](http://hl7.org/fhir/R4/extension-bodysite.html).</t>
-  </si>
-  <si>
-    <t>https://interoperabilidad.minsal.cl/fhir/ig/r2bo/ValueSet/r2bo-estructuras-anatomicas-VS</t>
-  </si>
-  <si>
-    <t>.targetSiteCode</t>
-  </si>
-  <si>
-    <t>SPM-8 and SPM-9</t>
-  </si>
-  <si>
-    <t>Specimen.collection.bodySite.id</t>
-  </si>
-  <si>
-    <t>Specimen.collection.bodySite.extension</t>
-  </si>
-  <si>
-    <t>Specimen.collection.bodySite.extension:CalificadorLateralidad</t>
-  </si>
-  <si>
-    <t>CalificadorLateralidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extension {http://hl7.org/fhir/us/mcode/StructureDefinition/mcode-laterality-qualifier}
-</t>
-  </si>
-  <si>
-    <t>Calificador para lateralidad para este sitio del cuerpo</t>
-  </si>
-  <si>
-    <t>Qualifier to specify laterality.</t>
-  </si>
-  <si>
-    <t>Specimen.collection.bodySite.coding</t>
-  </si>
-  <si>
-    <t>Specimen.collection.bodySite.text</t>
   </si>
   <si>
     <t>Specimen.collection.fastingStatus[x]</t>
@@ -1551,12 +1517,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AM59"/>
+  <dimension ref="A1:AM54"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="50.9453125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="50.84765625" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="32.90625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="19.1796875" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="3" max="3" width="18.40625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="34.8125" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.29296875" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.21484375" customWidth="true" bestFit="true"/>
@@ -1564,7 +1530,7 @@
     <col min="8" max="8" width="13.1171875" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="10.75390625" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="101.5234375" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="87.1484375" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -3605,7 +3571,7 @@
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="G19" t="s" s="2">
         <v>88</v>
@@ -4577,7 +4543,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="28" hidden="true">
+    <row r="28">
       <c r="A28" t="s" s="2">
         <v>255</v>
       </c>
@@ -4590,13 +4556,13 @@
       </c>
       <c r="E28" s="2"/>
       <c r="F28" t="s" s="2">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="G28" t="s" s="2">
         <v>88</v>
       </c>
       <c r="H28" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="I28" t="s" s="2">
         <v>79</v>
@@ -4605,15 +4571,17 @@
         <v>79</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>213</v>
+        <v>168</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>214</v>
+        <v>256</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>215</v>
-      </c>
-      <c r="N28" s="2"/>
+        <v>257</v>
+      </c>
+      <c r="N28" t="s" s="2">
+        <v>258</v>
+      </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
         <v>79</v>
@@ -4638,13 +4606,11 @@
         <v>79</v>
       </c>
       <c r="X28" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y28" t="s" s="2">
-        <v>79</v>
-      </c>
+        <v>172</v>
+      </c>
+      <c r="Y28" s="2"/>
       <c r="Z28" t="s" s="2">
-        <v>79</v>
+        <v>259</v>
       </c>
       <c r="AA28" t="s" s="2">
         <v>79</v>
@@ -4662,7 +4628,7 @@
         <v>79</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>216</v>
+        <v>255</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>80</v>
@@ -4674,24 +4640,24 @@
         <v>79</v>
       </c>
       <c r="AJ28" t="s" s="2">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>217</v>
+        <v>260</v>
       </c>
       <c r="AL28" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>79</v>
+        <v>261</v>
       </c>
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4699,11 +4665,11 @@
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="G29" t="s" s="2">
         <v>88</v>
       </c>
-      <c r="G29" t="s" s="2">
-        <v>81</v>
-      </c>
       <c r="H29" t="s" s="2">
         <v>79</v>
       </c>
@@ -4714,13 +4680,13 @@
         <v>79</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>134</v>
+        <v>213</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>257</v>
+        <v>214</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>258</v>
+        <v>215</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
@@ -4759,34 +4725,34 @@
         <v>79</v>
       </c>
       <c r="AB29" t="s" s="2">
-        <v>259</v>
+        <v>79</v>
       </c>
       <c r="AC29" t="s" s="2">
-        <v>260</v>
+        <v>79</v>
       </c>
       <c r="AD29" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE29" t="s" s="2">
-        <v>261</v>
+        <v>79</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH29" t="s" s="2">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="AI29" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ29" t="s" s="2">
-        <v>139</v>
+        <v>79</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>79</v>
+        <v>217</v>
       </c>
       <c r="AL29" t="s" s="2">
         <v>79</v>
@@ -4795,28 +4761,26 @@
         <v>79</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>256</v>
-      </c>
-      <c r="C30" t="s" s="2">
         <v>263</v>
       </c>
+      <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
-        <v>79</v>
+        <v>133</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="G30" t="s" s="2">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="H30" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="I30" t="s" s="2">
         <v>79</v>
@@ -4825,15 +4789,17 @@
         <v>79</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>264</v>
+        <v>134</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>265</v>
+        <v>135</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>266</v>
-      </c>
-      <c r="N30" s="2"/>
+        <v>219</v>
+      </c>
+      <c r="N30" t="s" s="2">
+        <v>137</v>
+      </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
         <v>79</v>
@@ -4870,16 +4836,16 @@
         <v>79</v>
       </c>
       <c r="AB30" t="s" s="2">
-        <v>79</v>
+        <v>264</v>
       </c>
       <c r="AC30" t="s" s="2">
-        <v>79</v>
+        <v>265</v>
       </c>
       <c r="AD30" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE30" t="s" s="2">
-        <v>79</v>
+        <v>266</v>
       </c>
       <c r="AF30" t="s" s="2">
         <v>220</v>
@@ -4897,7 +4863,7 @@
         <v>139</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>79</v>
+        <v>217</v>
       </c>
       <c r="AL30" t="s" s="2">
         <v>79</v>
@@ -4906,14 +4872,16 @@
         <v>79</v>
       </c>
     </row>
-    <row r="31" hidden="true">
+    <row r="31">
       <c r="A31" t="s" s="2">
         <v>267</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>267</v>
-      </c>
-      <c r="C31" s="2"/>
+        <v>263</v>
+      </c>
+      <c r="C31" t="s" s="2">
+        <v>268</v>
+      </c>
       <c r="D31" t="s" s="2">
         <v>79</v>
       </c>
@@ -4922,32 +4890,28 @@
         <v>80</v>
       </c>
       <c r="G31" t="s" s="2">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H31" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="I31" t="s" s="2">
         <v>79</v>
       </c>
       <c r="J31" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>270</v>
-      </c>
-      <c r="N31" t="s" s="2">
         <v>271</v>
       </c>
-      <c r="O31" t="s" s="2">
-        <v>272</v>
-      </c>
+      <c r="N31" s="2"/>
+      <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
         <v>79</v>
       </c>
@@ -4995,7 +4959,7 @@
         <v>79</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>273</v>
+        <v>220</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>80</v>
@@ -5007,24 +4971,24 @@
         <v>79</v>
       </c>
       <c r="AJ31" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>274</v>
+        <v>79</v>
       </c>
       <c r="AL31" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM31" t="s" s="2">
-        <v>275</v>
+        <v>79</v>
       </c>
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5035,7 +4999,7 @@
         <v>80</v>
       </c>
       <c r="G32" t="s" s="2">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="H32" t="s" s="2">
         <v>79</v>
@@ -5047,19 +5011,19 @@
         <v>89</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>213</v>
+        <v>273</v>
       </c>
       <c r="L32" t="s" s="2">
+        <v>274</v>
+      </c>
+      <c r="M32" t="s" s="2">
+        <v>275</v>
+      </c>
+      <c r="N32" t="s" s="2">
+        <v>276</v>
+      </c>
+      <c r="O32" t="s" s="2">
         <v>277</v>
-      </c>
-      <c r="M32" t="s" s="2">
-        <v>278</v>
-      </c>
-      <c r="N32" t="s" s="2">
-        <v>279</v>
-      </c>
-      <c r="O32" t="s" s="2">
-        <v>280</v>
       </c>
       <c r="P32" t="s" s="2">
         <v>79</v>
@@ -5108,13 +5072,13 @@
         <v>79</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH32" t="s" s="2">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="AI32" t="s" s="2">
         <v>79</v>
@@ -5123,21 +5087,21 @@
         <v>100</v>
       </c>
       <c r="AK32" t="s" s="2">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="AL32" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM32" t="s" s="2">
-        <v>283</v>
+        <v>280</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5145,33 +5109,35 @@
       </c>
       <c r="E33" s="2"/>
       <c r="F33" t="s" s="2">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="G33" t="s" s="2">
         <v>88</v>
       </c>
       <c r="H33" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="I33" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="J33" t="s" s="2">
         <v>89</v>
       </c>
-      <c r="I33" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J33" t="s" s="2">
-        <v>79</v>
-      </c>
       <c r="K33" t="s" s="2">
-        <v>168</v>
+        <v>213</v>
       </c>
       <c r="L33" t="s" s="2">
+        <v>282</v>
+      </c>
+      <c r="M33" t="s" s="2">
+        <v>283</v>
+      </c>
+      <c r="N33" t="s" s="2">
+        <v>284</v>
+      </c>
+      <c r="O33" t="s" s="2">
         <v>285</v>
       </c>
-      <c r="M33" t="s" s="2">
-        <v>286</v>
-      </c>
-      <c r="N33" t="s" s="2">
-        <v>287</v>
-      </c>
-      <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
         <v>79</v>
       </c>
@@ -5195,11 +5161,13 @@
         <v>79</v>
       </c>
       <c r="X33" t="s" s="2">
-        <v>172</v>
-      </c>
-      <c r="Y33" s="2"/>
+        <v>79</v>
+      </c>
+      <c r="Y33" t="s" s="2">
+        <v>79</v>
+      </c>
       <c r="Z33" t="s" s="2">
-        <v>288</v>
+        <v>79</v>
       </c>
       <c r="AA33" t="s" s="2">
         <v>79</v>
@@ -5217,7 +5185,7 @@
         <v>79</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>80</v>
@@ -5232,21 +5200,21 @@
         <v>100</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="AL33" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM33" t="s" s="2">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5266,19 +5234,23 @@
         <v>79</v>
       </c>
       <c r="J34" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>213</v>
+        <v>290</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>214</v>
+        <v>291</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>215</v>
-      </c>
-      <c r="N34" s="2"/>
-      <c r="O34" s="2"/>
+        <v>292</v>
+      </c>
+      <c r="N34" t="s" s="2">
+        <v>293</v>
+      </c>
+      <c r="O34" t="s" s="2">
+        <v>294</v>
+      </c>
       <c r="P34" t="s" s="2">
         <v>79</v>
       </c>
@@ -5302,13 +5274,11 @@
         <v>79</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y34" t="s" s="2">
-        <v>79</v>
-      </c>
+        <v>172</v>
+      </c>
+      <c r="Y34" s="2"/>
       <c r="Z34" t="s" s="2">
-        <v>79</v>
+        <v>295</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>79</v>
@@ -5326,7 +5296,7 @@
         <v>79</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>216</v>
+        <v>289</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>80</v>
@@ -5338,28 +5308,28 @@
         <v>79</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>217</v>
+        <v>79</v>
       </c>
       <c r="AL34" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>79</v>
+        <v>296</v>
       </c>
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
-        <v>133</v>
+        <v>79</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
@@ -5378,17 +5348,15 @@
         <v>79</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>134</v>
+        <v>207</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>135</v>
+        <v>298</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>219</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>137</v>
-      </c>
+        <v>299</v>
+      </c>
+      <c r="N35" s="2"/>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
         <v>79</v>
@@ -5425,19 +5393,19 @@
         <v>79</v>
       </c>
       <c r="AB35" t="s" s="2">
-        <v>259</v>
+        <v>79</v>
       </c>
       <c r="AC35" t="s" s="2">
-        <v>260</v>
+        <v>79</v>
       </c>
       <c r="AD35" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AE35" t="s" s="2">
-        <v>261</v>
+        <v>79</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>220</v>
+        <v>297</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>80</v>
@@ -5449,10 +5417,10 @@
         <v>79</v>
       </c>
       <c r="AJ35" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>217</v>
+        <v>300</v>
       </c>
       <c r="AL35" t="s" s="2">
         <v>79</v>
@@ -5461,16 +5429,14 @@
         <v>79</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>292</v>
-      </c>
-      <c r="C36" t="s" s="2">
-        <v>294</v>
-      </c>
+        <v>301</v>
+      </c>
+      <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
         <v>79</v>
       </c>
@@ -5482,7 +5448,7 @@
         <v>88</v>
       </c>
       <c r="H36" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="I36" t="s" s="2">
         <v>79</v>
@@ -5491,13 +5457,13 @@
         <v>79</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>295</v>
+        <v>213</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>296</v>
+        <v>214</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>297</v>
+        <v>215</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -5548,22 +5514,22 @@
         <v>79</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH36" t="s" s="2">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="AI36" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ36" t="s" s="2">
-        <v>139</v>
+        <v>79</v>
       </c>
       <c r="AK36" t="s" s="2">
-        <v>79</v>
+        <v>217</v>
       </c>
       <c r="AL36" t="s" s="2">
         <v>79</v>
@@ -5574,14 +5540,14 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>298</v>
+        <v>302</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>79</v>
+        <v>133</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
@@ -5597,23 +5563,21 @@
         <v>79</v>
       </c>
       <c r="J37" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>268</v>
+        <v>134</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>269</v>
+        <v>135</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>270</v>
+        <v>219</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>271</v>
-      </c>
-      <c r="O37" t="s" s="2">
-        <v>272</v>
-      </c>
+        <v>137</v>
+      </c>
+      <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
         <v>79</v>
       </c>
@@ -5661,7 +5625,7 @@
         <v>79</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>273</v>
+        <v>220</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>80</v>
@@ -5673,59 +5637,59 @@
         <v>79</v>
       </c>
       <c r="AJ37" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK37" t="s" s="2">
-        <v>274</v>
+        <v>217</v>
       </c>
       <c r="AL37" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM37" t="s" s="2">
-        <v>275</v>
+        <v>79</v>
       </c>
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>299</v>
+        <v>303</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
-        <v>79</v>
+        <v>222</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G38" t="s" s="2">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="H38" t="s" s="2">
         <v>79</v>
       </c>
       <c r="I38" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="J38" t="s" s="2">
         <v>89</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>213</v>
+        <v>134</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>277</v>
+        <v>223</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>278</v>
+        <v>224</v>
       </c>
       <c r="N38" t="s" s="2">
-        <v>279</v>
+        <v>137</v>
       </c>
       <c r="O38" t="s" s="2">
-        <v>280</v>
+        <v>143</v>
       </c>
       <c r="P38" t="s" s="2">
         <v>79</v>
@@ -5774,36 +5738,36 @@
         <v>79</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>281</v>
+        <v>225</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH38" t="s" s="2">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="AI38" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ38" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK38" t="s" s="2">
-        <v>282</v>
+        <v>131</v>
       </c>
       <c r="AL38" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>283</v>
+        <v>79</v>
       </c>
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5823,23 +5787,19 @@
         <v>79</v>
       </c>
       <c r="J39" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>301</v>
+        <v>213</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>303</v>
-      </c>
-      <c r="N39" t="s" s="2">
-        <v>304</v>
-      </c>
-      <c r="O39" t="s" s="2">
-        <v>305</v>
-      </c>
+        <v>306</v>
+      </c>
+      <c r="N39" s="2"/>
+      <c r="O39" s="2"/>
       <c r="P39" t="s" s="2">
         <v>79</v>
       </c>
@@ -5863,11 +5823,13 @@
         <v>79</v>
       </c>
       <c r="X39" t="s" s="2">
-        <v>172</v>
-      </c>
-      <c r="Y39" s="2"/>
+        <v>79</v>
+      </c>
+      <c r="Y39" t="s" s="2">
+        <v>79</v>
+      </c>
       <c r="Z39" t="s" s="2">
-        <v>306</v>
+        <v>79</v>
       </c>
       <c r="AA39" t="s" s="2">
         <v>79</v>
@@ -5885,7 +5847,7 @@
         <v>79</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>80</v>
@@ -5900,13 +5862,13 @@
         <v>100</v>
       </c>
       <c r="AK39" t="s" s="2">
-        <v>79</v>
+        <v>307</v>
       </c>
       <c r="AL39" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM39" t="s" s="2">
-        <v>307</v>
+        <v>79</v>
       </c>
     </row>
     <row r="40" hidden="true">
@@ -5925,7 +5887,7 @@
         <v>80</v>
       </c>
       <c r="G40" t="s" s="2">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H40" t="s" s="2">
         <v>79</v>
@@ -5937,7 +5899,7 @@
         <v>79</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>207</v>
+        <v>168</v>
       </c>
       <c r="L40" t="s" s="2">
         <v>309</v>
@@ -5970,13 +5932,13 @@
         <v>79</v>
       </c>
       <c r="X40" t="s" s="2">
-        <v>79</v>
+        <v>311</v>
       </c>
       <c r="Y40" t="s" s="2">
-        <v>79</v>
+        <v>312</v>
       </c>
       <c r="Z40" t="s" s="2">
-        <v>79</v>
+        <v>313</v>
       </c>
       <c r="AA40" t="s" s="2">
         <v>79</v>
@@ -6000,7 +5962,7 @@
         <v>80</v>
       </c>
       <c r="AH40" t="s" s="2">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="AI40" t="s" s="2">
         <v>79</v>
@@ -6009,7 +5971,7 @@
         <v>100</v>
       </c>
       <c r="AK40" t="s" s="2">
-        <v>311</v>
+        <v>175</v>
       </c>
       <c r="AL40" t="s" s="2">
         <v>79</v>
@@ -6020,10 +5982,10 @@
     </row>
     <row r="41" hidden="true">
       <c r="A41" t="s" s="2">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6034,7 +5996,7 @@
         <v>80</v>
       </c>
       <c r="G41" t="s" s="2">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="H41" t="s" s="2">
         <v>79</v>
@@ -6046,13 +6008,13 @@
         <v>79</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>213</v>
+        <v>315</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>214</v>
+        <v>316</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>215</v>
+        <v>317</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -6103,47 +6065,47 @@
         <v>79</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>216</v>
+        <v>314</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH41" t="s" s="2">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="AI41" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ41" t="s" s="2">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="AK41" t="s" s="2">
-        <v>217</v>
+        <v>318</v>
       </c>
       <c r="AL41" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM41" t="s" s="2">
-        <v>79</v>
+        <v>319</v>
       </c>
     </row>
     <row r="42" hidden="true">
       <c r="A42" t="s" s="2">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
-        <v>133</v>
+        <v>79</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G42" t="s" s="2">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H42" t="s" s="2">
         <v>79</v>
@@ -6155,17 +6117,15 @@
         <v>79</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>134</v>
+        <v>321</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>135</v>
+        <v>322</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>219</v>
-      </c>
-      <c r="N42" t="s" s="2">
-        <v>137</v>
-      </c>
+        <v>323</v>
+      </c>
+      <c r="N42" s="2"/>
       <c r="O42" s="2"/>
       <c r="P42" t="s" s="2">
         <v>79</v>
@@ -6214,22 +6174,22 @@
         <v>79</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>220</v>
+        <v>320</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH42" t="s" s="2">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="AI42" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK42" t="s" s="2">
-        <v>217</v>
+        <v>236</v>
       </c>
       <c r="AL42" t="s" s="2">
         <v>79</v>
@@ -6240,14 +6200,14 @@
     </row>
     <row r="43" hidden="true">
       <c r="A43" t="s" s="2">
-        <v>314</v>
+        <v>324</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>314</v>
+        <v>324</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>222</v>
+        <v>79</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
@@ -6260,26 +6220,22 @@
         <v>79</v>
       </c>
       <c r="I43" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="J43" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>134</v>
+        <v>207</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>223</v>
+        <v>325</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>224</v>
-      </c>
-      <c r="N43" t="s" s="2">
-        <v>137</v>
-      </c>
-      <c r="O43" t="s" s="2">
-        <v>143</v>
-      </c>
+        <v>326</v>
+      </c>
+      <c r="N43" s="2"/>
+      <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
         <v>79</v>
       </c>
@@ -6327,7 +6283,7 @@
         <v>79</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>225</v>
+        <v>324</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>80</v>
@@ -6339,10 +6295,10 @@
         <v>79</v>
       </c>
       <c r="AJ43" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK43" t="s" s="2">
-        <v>131</v>
+        <v>327</v>
       </c>
       <c r="AL43" t="s" s="2">
         <v>79</v>
@@ -6353,10 +6309,10 @@
     </row>
     <row r="44" hidden="true">
       <c r="A44" t="s" s="2">
-        <v>315</v>
+        <v>328</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>315</v>
+        <v>328</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -6382,10 +6338,10 @@
         <v>213</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>316</v>
+        <v>214</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>317</v>
+        <v>215</v>
       </c>
       <c r="N44" s="2"/>
       <c r="O44" s="2"/>
@@ -6436,7 +6392,7 @@
         <v>79</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>315</v>
+        <v>216</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>80</v>
@@ -6448,10 +6404,10 @@
         <v>79</v>
       </c>
       <c r="AJ44" t="s" s="2">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="AK44" t="s" s="2">
-        <v>318</v>
+        <v>217</v>
       </c>
       <c r="AL44" t="s" s="2">
         <v>79</v>
@@ -6462,21 +6418,21 @@
     </row>
     <row r="45" hidden="true">
       <c r="A45" t="s" s="2">
-        <v>319</v>
+        <v>329</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>319</v>
+        <v>329</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
-        <v>79</v>
+        <v>133</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G45" t="s" s="2">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="H45" t="s" s="2">
         <v>79</v>
@@ -6488,15 +6444,17 @@
         <v>79</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>168</v>
+        <v>134</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>320</v>
+        <v>135</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>321</v>
-      </c>
-      <c r="N45" s="2"/>
+        <v>219</v>
+      </c>
+      <c r="N45" t="s" s="2">
+        <v>137</v>
+      </c>
       <c r="O45" s="2"/>
       <c r="P45" t="s" s="2">
         <v>79</v>
@@ -6521,13 +6479,13 @@
         <v>79</v>
       </c>
       <c r="X45" t="s" s="2">
-        <v>322</v>
+        <v>79</v>
       </c>
       <c r="Y45" t="s" s="2">
-        <v>323</v>
+        <v>79</v>
       </c>
       <c r="Z45" t="s" s="2">
-        <v>324</v>
+        <v>79</v>
       </c>
       <c r="AA45" t="s" s="2">
         <v>79</v>
@@ -6545,22 +6503,22 @@
         <v>79</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>319</v>
+        <v>220</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH45" t="s" s="2">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="AI45" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ45" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK45" t="s" s="2">
-        <v>175</v>
+        <v>217</v>
       </c>
       <c r="AL45" t="s" s="2">
         <v>79</v>
@@ -6571,14 +6529,14 @@
     </row>
     <row r="46" hidden="true">
       <c r="A46" t="s" s="2">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
-        <v>79</v>
+        <v>222</v>
       </c>
       <c r="E46" s="2"/>
       <c r="F46" t="s" s="2">
@@ -6591,22 +6549,26 @@
         <v>79</v>
       </c>
       <c r="I46" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="J46" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>326</v>
+        <v>134</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>327</v>
+        <v>223</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>328</v>
-      </c>
-      <c r="N46" s="2"/>
-      <c r="O46" s="2"/>
+        <v>224</v>
+      </c>
+      <c r="N46" t="s" s="2">
+        <v>137</v>
+      </c>
+      <c r="O46" t="s" s="2">
+        <v>143</v>
+      </c>
       <c r="P46" t="s" s="2">
         <v>79</v>
       </c>
@@ -6654,7 +6616,7 @@
         <v>79</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>325</v>
+        <v>225</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>80</v>
@@ -6666,16 +6628,16 @@
         <v>79</v>
       </c>
       <c r="AJ46" t="s" s="2">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="AK46" t="s" s="2">
-        <v>329</v>
+        <v>131</v>
       </c>
       <c r="AL46" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM46" t="s" s="2">
-        <v>330</v>
+        <v>79</v>
       </c>
     </row>
     <row r="47" hidden="true">
@@ -6694,7 +6656,7 @@
         <v>80</v>
       </c>
       <c r="G47" t="s" s="2">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="H47" t="s" s="2">
         <v>79</v>
@@ -6703,16 +6665,16 @@
         <v>79</v>
       </c>
       <c r="J47" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="K47" t="s" s="2">
+        <v>146</v>
+      </c>
+      <c r="L47" t="s" s="2">
         <v>332</v>
       </c>
-      <c r="L47" t="s" s="2">
+      <c r="M47" t="s" s="2">
         <v>333</v>
-      </c>
-      <c r="M47" t="s" s="2">
-        <v>334</v>
       </c>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
@@ -6769,7 +6731,7 @@
         <v>80</v>
       </c>
       <c r="AH47" t="s" s="2">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="AI47" t="s" s="2">
         <v>79</v>
@@ -6778,13 +6740,13 @@
         <v>100</v>
       </c>
       <c r="AK47" t="s" s="2">
-        <v>236</v>
+        <v>149</v>
       </c>
       <c r="AL47" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM47" t="s" s="2">
-        <v>79</v>
+        <v>334</v>
       </c>
     </row>
     <row r="48" hidden="true">
@@ -6803,7 +6765,7 @@
         <v>80</v>
       </c>
       <c r="G48" t="s" s="2">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H48" t="s" s="2">
         <v>79</v>
@@ -6815,7 +6777,7 @@
         <v>79</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="L48" t="s" s="2">
         <v>336</v>
@@ -6878,7 +6840,7 @@
         <v>80</v>
       </c>
       <c r="AH48" t="s" s="2">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="AI48" t="s" s="2">
         <v>79</v>
@@ -6924,13 +6886,13 @@
         <v>79</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>213</v>
+        <v>168</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>214</v>
+        <v>340</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>215</v>
+        <v>341</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
@@ -6957,13 +6919,13 @@
         <v>79</v>
       </c>
       <c r="X49" t="s" s="2">
-        <v>79</v>
+        <v>311</v>
       </c>
       <c r="Y49" t="s" s="2">
-        <v>79</v>
+        <v>342</v>
       </c>
       <c r="Z49" t="s" s="2">
-        <v>79</v>
+        <v>343</v>
       </c>
       <c r="AA49" t="s" s="2">
         <v>79</v>
@@ -6981,7 +6943,7 @@
         <v>79</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>216</v>
+        <v>339</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>80</v>
@@ -6993,35 +6955,35 @@
         <v>79</v>
       </c>
       <c r="AJ49" t="s" s="2">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="AK49" t="s" s="2">
-        <v>217</v>
+        <v>175</v>
       </c>
       <c r="AL49" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM49" t="s" s="2">
-        <v>79</v>
+        <v>344</v>
       </c>
     </row>
     <row r="50" hidden="true">
       <c r="A50" t="s" s="2">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
-        <v>133</v>
+        <v>79</v>
       </c>
       <c r="E50" s="2"/>
       <c r="F50" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G50" t="s" s="2">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H50" t="s" s="2">
         <v>79</v>
@@ -7033,17 +6995,15 @@
         <v>79</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>134</v>
+        <v>244</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>135</v>
+        <v>346</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>219</v>
-      </c>
-      <c r="N50" t="s" s="2">
-        <v>137</v>
-      </c>
+        <v>347</v>
+      </c>
+      <c r="N50" s="2"/>
       <c r="O50" s="2"/>
       <c r="P50" t="s" s="2">
         <v>79</v>
@@ -7092,72 +7052,68 @@
         <v>79</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>220</v>
+        <v>345</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH50" t="s" s="2">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="AI50" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ50" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK50" t="s" s="2">
-        <v>217</v>
+        <v>348</v>
       </c>
       <c r="AL50" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM50" t="s" s="2">
-        <v>79</v>
+        <v>349</v>
       </c>
     </row>
     <row r="51" hidden="true">
       <c r="A51" t="s" s="2">
-        <v>341</v>
+        <v>350</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>341</v>
+        <v>350</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
-        <v>222</v>
+        <v>79</v>
       </c>
       <c r="E51" s="2"/>
       <c r="F51" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G51" t="s" s="2">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H51" t="s" s="2">
         <v>79</v>
       </c>
       <c r="I51" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="J51" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>134</v>
+        <v>244</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>223</v>
+        <v>351</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>224</v>
-      </c>
-      <c r="N51" t="s" s="2">
-        <v>137</v>
-      </c>
-      <c r="O51" t="s" s="2">
-        <v>143</v>
-      </c>
+        <v>352</v>
+      </c>
+      <c r="N51" s="2"/>
+      <c r="O51" s="2"/>
       <c r="P51" t="s" s="2">
         <v>79</v>
       </c>
@@ -7205,36 +7161,36 @@
         <v>79</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>225</v>
+        <v>350</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH51" t="s" s="2">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="AI51" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AJ51" t="s" s="2">
-        <v>139</v>
+        <v>100</v>
       </c>
       <c r="AK51" t="s" s="2">
-        <v>131</v>
+        <v>353</v>
       </c>
       <c r="AL51" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM51" t="s" s="2">
-        <v>79</v>
+        <v>354</v>
       </c>
     </row>
     <row r="52" hidden="true">
       <c r="A52" t="s" s="2">
-        <v>342</v>
+        <v>355</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>342</v>
+        <v>355</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -7245,7 +7201,7 @@
         <v>80</v>
       </c>
       <c r="G52" t="s" s="2">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="H52" t="s" s="2">
         <v>79</v>
@@ -7254,16 +7210,16 @@
         <v>79</v>
       </c>
       <c r="J52" t="s" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>146</v>
+        <v>356</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>343</v>
+        <v>357</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>344</v>
+        <v>358</v>
       </c>
       <c r="N52" s="2"/>
       <c r="O52" s="2"/>
@@ -7290,13 +7246,13 @@
         <v>79</v>
       </c>
       <c r="X52" t="s" s="2">
-        <v>79</v>
+        <v>311</v>
       </c>
       <c r="Y52" t="s" s="2">
-        <v>79</v>
+        <v>359</v>
       </c>
       <c r="Z52" t="s" s="2">
-        <v>79</v>
+        <v>360</v>
       </c>
       <c r="AA52" t="s" s="2">
         <v>79</v>
@@ -7314,13 +7270,13 @@
         <v>79</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>342</v>
+        <v>355</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH52" t="s" s="2">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="AI52" t="s" s="2">
         <v>79</v>
@@ -7329,21 +7285,21 @@
         <v>100</v>
       </c>
       <c r="AK52" t="s" s="2">
-        <v>149</v>
+        <v>361</v>
       </c>
       <c r="AL52" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM52" t="s" s="2">
-        <v>345</v>
+        <v>362</v>
       </c>
     </row>
     <row r="53" hidden="true">
       <c r="A53" t="s" s="2">
-        <v>346</v>
+        <v>363</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>346</v>
+        <v>363</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -7354,7 +7310,7 @@
         <v>80</v>
       </c>
       <c r="G53" t="s" s="2">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="H53" t="s" s="2">
         <v>79</v>
@@ -7363,19 +7319,23 @@
         <v>79</v>
       </c>
       <c r="J53" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>213</v>
+        <v>168</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>347</v>
+        <v>364</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>348</v>
-      </c>
-      <c r="N53" s="2"/>
-      <c r="O53" s="2"/>
+        <v>365</v>
+      </c>
+      <c r="N53" t="s" s="2">
+        <v>366</v>
+      </c>
+      <c r="O53" t="s" s="2">
+        <v>367</v>
+      </c>
       <c r="P53" t="s" s="2">
         <v>79</v>
       </c>
@@ -7399,13 +7359,13 @@
         <v>79</v>
       </c>
       <c r="X53" t="s" s="2">
-        <v>79</v>
+        <v>172</v>
       </c>
       <c r="Y53" t="s" s="2">
-        <v>79</v>
+        <v>368</v>
       </c>
       <c r="Z53" t="s" s="2">
-        <v>79</v>
+        <v>369</v>
       </c>
       <c r="AA53" t="s" s="2">
         <v>79</v>
@@ -7423,13 +7383,13 @@
         <v>79</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>346</v>
+        <v>363</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH53" t="s" s="2">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="AI53" t="s" s="2">
         <v>79</v>
@@ -7438,21 +7398,21 @@
         <v>100</v>
       </c>
       <c r="AK53" t="s" s="2">
-        <v>349</v>
+        <v>79</v>
       </c>
       <c r="AL53" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM53" t="s" s="2">
-        <v>79</v>
+        <v>370</v>
       </c>
     </row>
-    <row r="54" hidden="true">
+    <row r="54">
       <c r="A54" t="s" s="2">
-        <v>350</v>
+        <v>371</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>350</v>
+        <v>371</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -7463,10 +7423,10 @@
         <v>80</v>
       </c>
       <c r="G54" t="s" s="2">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="H54" t="s" s="2">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="I54" t="s" s="2">
         <v>79</v>
@@ -7475,13 +7435,13 @@
         <v>79</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>168</v>
+        <v>372</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>351</v>
+        <v>373</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>352</v>
+        <v>374</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
@@ -7508,13 +7468,13 @@
         <v>79</v>
       </c>
       <c r="X54" t="s" s="2">
-        <v>322</v>
+        <v>79</v>
       </c>
       <c r="Y54" t="s" s="2">
-        <v>353</v>
+        <v>79</v>
       </c>
       <c r="Z54" t="s" s="2">
-        <v>354</v>
+        <v>79</v>
       </c>
       <c r="AA54" t="s" s="2">
         <v>79</v>
@@ -7532,13 +7492,13 @@
         <v>79</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>350</v>
+        <v>371</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>80</v>
       </c>
       <c r="AH54" t="s" s="2">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="AI54" t="s" s="2">
         <v>79</v>
@@ -7547,566 +7507,17 @@
         <v>100</v>
       </c>
       <c r="AK54" t="s" s="2">
-        <v>175</v>
+        <v>375</v>
       </c>
       <c r="AL54" t="s" s="2">
         <v>79</v>
       </c>
       <c r="AM54" t="s" s="2">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="55" hidden="true">
-      <c r="A55" t="s" s="2">
-        <v>356</v>
-      </c>
-      <c r="B55" t="s" s="2">
-        <v>356</v>
-      </c>
-      <c r="C55" s="2"/>
-      <c r="D55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E55" s="2"/>
-      <c r="F55" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G55" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="H55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K55" t="s" s="2">
-        <v>244</v>
-      </c>
-      <c r="L55" t="s" s="2">
-        <v>357</v>
-      </c>
-      <c r="M55" t="s" s="2">
-        <v>358</v>
-      </c>
-      <c r="N55" s="2"/>
-      <c r="O55" s="2"/>
-      <c r="P55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q55" s="2"/>
-      <c r="R55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF55" t="s" s="2">
-        <v>356</v>
-      </c>
-      <c r="AG55" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH55" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AI55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AJ55" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK55" t="s" s="2">
-        <v>359</v>
-      </c>
-      <c r="AL55" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM55" t="s" s="2">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="56" hidden="true">
-      <c r="A56" t="s" s="2">
-        <v>361</v>
-      </c>
-      <c r="B56" t="s" s="2">
-        <v>361</v>
-      </c>
-      <c r="C56" s="2"/>
-      <c r="D56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E56" s="2"/>
-      <c r="F56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G56" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="H56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K56" t="s" s="2">
-        <v>244</v>
-      </c>
-      <c r="L56" t="s" s="2">
-        <v>362</v>
-      </c>
-      <c r="M56" t="s" s="2">
-        <v>363</v>
-      </c>
-      <c r="N56" s="2"/>
-      <c r="O56" s="2"/>
-      <c r="P56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q56" s="2"/>
-      <c r="R56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF56" t="s" s="2">
-        <v>361</v>
-      </c>
-      <c r="AG56" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH56" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AI56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AJ56" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK56" t="s" s="2">
-        <v>364</v>
-      </c>
-      <c r="AL56" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM56" t="s" s="2">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="57" hidden="true">
-      <c r="A57" t="s" s="2">
-        <v>366</v>
-      </c>
-      <c r="B57" t="s" s="2">
-        <v>366</v>
-      </c>
-      <c r="C57" s="2"/>
-      <c r="D57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E57" s="2"/>
-      <c r="F57" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G57" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="H57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K57" t="s" s="2">
-        <v>367</v>
-      </c>
-      <c r="L57" t="s" s="2">
-        <v>368</v>
-      </c>
-      <c r="M57" t="s" s="2">
-        <v>369</v>
-      </c>
-      <c r="N57" s="2"/>
-      <c r="O57" s="2"/>
-      <c r="P57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q57" s="2"/>
-      <c r="R57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X57" t="s" s="2">
-        <v>322</v>
-      </c>
-      <c r="Y57" t="s" s="2">
-        <v>370</v>
-      </c>
-      <c r="Z57" t="s" s="2">
-        <v>371</v>
-      </c>
-      <c r="AA57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF57" t="s" s="2">
-        <v>366</v>
-      </c>
-      <c r="AG57" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH57" t="s" s="2">
-        <v>88</v>
-      </c>
-      <c r="AI57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AJ57" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK57" t="s" s="2">
-        <v>372</v>
-      </c>
-      <c r="AL57" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM57" t="s" s="2">
-        <v>373</v>
-      </c>
-    </row>
-    <row r="58" hidden="true">
-      <c r="A58" t="s" s="2">
-        <v>374</v>
-      </c>
-      <c r="B58" t="s" s="2">
-        <v>374</v>
-      </c>
-      <c r="C58" s="2"/>
-      <c r="D58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E58" s="2"/>
-      <c r="F58" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G58" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="I58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J58" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="K58" t="s" s="2">
-        <v>168</v>
-      </c>
-      <c r="L58" t="s" s="2">
-        <v>375</v>
-      </c>
-      <c r="M58" t="s" s="2">
         <v>376</v>
-      </c>
-      <c r="N58" t="s" s="2">
-        <v>377</v>
-      </c>
-      <c r="O58" t="s" s="2">
-        <v>378</v>
-      </c>
-      <c r="P58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q58" s="2"/>
-      <c r="R58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X58" t="s" s="2">
-        <v>172</v>
-      </c>
-      <c r="Y58" t="s" s="2">
-        <v>379</v>
-      </c>
-      <c r="Z58" t="s" s="2">
-        <v>380</v>
-      </c>
-      <c r="AA58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF58" t="s" s="2">
-        <v>374</v>
-      </c>
-      <c r="AG58" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH58" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AJ58" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AL58" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM58" t="s" s="2">
-        <v>381</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="s" s="2">
-        <v>382</v>
-      </c>
-      <c r="B59" t="s" s="2">
-        <v>382</v>
-      </c>
-      <c r="C59" s="2"/>
-      <c r="D59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="E59" s="2"/>
-      <c r="F59" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="G59" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H59" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="I59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="J59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="K59" t="s" s="2">
-        <v>383</v>
-      </c>
-      <c r="L59" t="s" s="2">
-        <v>384</v>
-      </c>
-      <c r="M59" t="s" s="2">
-        <v>385</v>
-      </c>
-      <c r="N59" s="2"/>
-      <c r="O59" s="2"/>
-      <c r="P59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Q59" s="2"/>
-      <c r="R59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="S59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="T59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="U59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="V59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="W59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="X59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Y59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="Z59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AA59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AB59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AC59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AD59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AE59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AF59" t="s" s="2">
-        <v>382</v>
-      </c>
-      <c r="AG59" t="s" s="2">
-        <v>80</v>
-      </c>
-      <c r="AH59" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AJ59" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="AK59" t="s" s="2">
-        <v>386</v>
-      </c>
-      <c r="AL59" t="s" s="2">
-        <v>79</v>
-      </c>
-      <c r="AM59" t="s" s="2">
-        <v>387</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AM59">
+  <autoFilter ref="A1:AM54">
     <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
@@ -8116,7 +7527,7 @@
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>
-  <conditionalFormatting sqref="A2:AI58">
+  <conditionalFormatting sqref="A2:AI53">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$G2&lt;&gt;"Y"</formula>
     </cfRule>

</xml_diff>